<commit_message>
feat: add request date display and rejection reason input
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/로그인정보.xlsx
+++ b/로그인정보.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\사무용품-신청-싸이트\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A9CA2AF-F28F-49D5-A47A-1767BBD29341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC38B02-C6A4-4D5A-8CEB-EEE73EFD15C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateCount="1"/>
+  <calcPr calcId="191029" iterateCount="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t>사번</t>
   </si>
@@ -299,6 +312,10 @@
   </si>
   <si>
     <t>김도연</t>
+  </si>
+  <si>
+    <t>비밀번호</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -775,745 +792,1021 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B92"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="9.3984375" customWidth="1"/>
+    <col min="1" max="3" width="9.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>240009</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="2">
+        <v>240009</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>120002</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="2">
+        <v>120002</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>230006</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="2">
+        <v>230006</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>250008</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="2">
+        <v>250008</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>120032</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="2">
+        <v>120032</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>110007</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="2">
+        <v>110007</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>110035</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="2">
+        <v>110035</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>120005</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="2">
+        <v>120005</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>110010</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="2">
+        <v>110010</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>130007</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="2">
+        <v>130007</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>160002</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="2">
+        <v>160002</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>200018</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="2">
+        <v>200018</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>130013</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="2">
+        <v>130013</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>140002</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="2">
+        <v>140002</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
         <v>140006</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="2">
+        <v>140006</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" s="2">
         <v>200012</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="2">
+        <v>200012</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" s="2">
         <v>250001</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="2">
+        <v>250001</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="2">
         <v>250007</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="2">
+        <v>250007</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="2">
         <v>160005</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="2">
+        <v>160005</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="2">
         <v>220008</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="2">
+        <v>220008</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="2">
         <v>180006</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="2">
+        <v>180006</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="2">
         <v>120006</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="2">
+        <v>120006</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="2">
         <v>110038</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="2">
+        <v>110038</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="2">
         <v>140009</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="2">
+        <v>140009</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" s="2">
         <v>120017</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="2">
+        <v>120017</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" s="2">
         <v>180007</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="2">
+        <v>180007</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="2">
         <v>230002</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="2">
+        <v>230002</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="2">
         <v>240001</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="2">
+        <v>240001</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="2">
         <v>110022</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="2">
+        <v>110022</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="2">
         <v>250002</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="2">
+        <v>250002</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="2">
         <v>160004</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="2">
+        <v>160004</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="2">
         <v>170007</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="2">
+        <v>170007</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="2">
         <v>240007</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="2">
+        <v>240007</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="2">
         <v>150002</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="2">
+        <v>150002</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="2">
         <v>150011</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="2">
+        <v>150011</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="2">
         <v>110046</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="2">
+        <v>110046</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="2">
         <v>120039</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="2">
+        <v>120039</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A39" s="2">
         <v>130011</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="2">
+        <v>130011</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A40" s="2">
         <v>170002</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="2">
+        <v>170002</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A41" s="2">
         <v>210015</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="2">
+        <v>210015</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" s="2">
         <v>240002</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="2">
+        <v>240002</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A43" s="2">
         <v>130006</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="2">
+        <v>130006</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A44" s="2">
         <v>120019</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="2">
+        <v>120019</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A45" s="2">
         <v>120036</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="2">
+        <v>120036</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A46" s="2">
         <v>170009</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="2">
+        <v>170009</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A47" s="2">
         <v>240005</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="2">
+        <v>240005</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A48" s="2">
         <v>170003</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="2">
+        <v>170003</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A49" s="2">
         <v>240006</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="2">
+        <v>240006</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A50" s="2">
         <v>240003</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="2">
+        <v>240003</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A51" s="2">
         <v>240004</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="2">
+        <v>240004</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A52" s="2">
         <v>130010</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="2">
+        <v>130010</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A53" s="2">
         <v>200014</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="2">
+        <v>200014</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A54" s="2">
         <v>220005</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="2">
+        <v>220005</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A55" s="2">
         <v>130003</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="2">
+        <v>130003</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A56" s="2">
         <v>130005</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="2">
+        <v>130005</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A57" s="2">
         <v>160003</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="2">
+        <v>160003</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A58" s="2">
         <v>150009</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="2">
+        <v>150009</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A59" s="2">
         <v>170006</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" s="2">
+        <v>170006</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A60" s="2">
         <v>210014</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="2">
+        <v>210014</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A61" s="2">
         <v>250003</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="2">
+        <v>250003</v>
+      </c>
+      <c r="C61" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A62" s="2">
         <v>110023</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="2">
+        <v>110023</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A63" s="2">
         <v>120023</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" s="2">
+        <v>120023</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A64" s="2">
         <v>120018</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="2">
+        <v>120018</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A65" s="2">
         <v>110011</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="2">
+        <v>110011</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A66" s="2">
         <v>120034</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="2">
+        <v>120034</v>
+      </c>
+      <c r="C66" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A67" s="2">
         <v>110039</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="2">
+        <v>110039</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A68" s="2">
         <v>210016</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="2">
+        <v>210016</v>
+      </c>
+      <c r="C68" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A69" s="2">
         <v>140004</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="2">
+        <v>140004</v>
+      </c>
+      <c r="C69" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A70" s="2">
         <v>240008</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="2">
+        <v>240008</v>
+      </c>
+      <c r="C70" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A71" s="2">
         <v>210013</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="2">
+        <v>210013</v>
+      </c>
+      <c r="C71" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A72" s="2">
         <v>220006</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" s="2">
+        <v>220006</v>
+      </c>
+      <c r="C72" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A73" s="2">
         <v>120003</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" s="2">
+        <v>120003</v>
+      </c>
+      <c r="C73" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A74" s="2">
         <v>140012</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="2">
+        <v>140012</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A75" s="2">
         <v>130001</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" s="2">
+        <v>130001</v>
+      </c>
+      <c r="C75" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A76" s="2">
         <v>120040</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" s="2">
+        <v>120040</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A77" s="2">
         <v>130002</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" s="2">
+        <v>130002</v>
+      </c>
+      <c r="C77" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A78" s="2">
         <v>120014</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" s="2">
+        <v>120014</v>
+      </c>
+      <c r="C78" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A79" s="2">
         <v>120042</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" s="2">
+        <v>120042</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A80" s="2">
         <v>120041</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B80" s="2">
+        <v>120041</v>
+      </c>
+      <c r="C80" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A81" s="2">
         <v>120029</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="B81" s="2">
+        <v>120029</v>
+      </c>
+      <c r="C81" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A82" s="2">
         <v>250005</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" s="2">
+        <v>250005</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A83" s="2">
         <v>120044</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B83" s="2">
+        <v>120044</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A84" s="2">
         <v>190002</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B84" s="2">
+        <v>190002</v>
+      </c>
+      <c r="C84" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A85" s="2">
         <v>220004</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B85" s="2">
+        <v>220004</v>
+      </c>
+      <c r="C85" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A86" s="2">
         <v>250006</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B86" s="2">
+        <v>250006</v>
+      </c>
+      <c r="C86" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A87" s="2">
         <v>250004</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="B87" s="2">
+        <v>250004</v>
+      </c>
+      <c r="C87" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A88" s="3">
         <v>500133</v>
       </c>
-      <c r="B88" s="3" t="s">
+      <c r="B88" s="3">
+        <v>500133</v>
+      </c>
+      <c r="C88" s="3" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A89" s="3">
         <v>500124</v>
       </c>
-      <c r="B89" s="3" t="s">
+      <c r="B89" s="3">
+        <v>500124</v>
+      </c>
+      <c r="C89" s="3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A90" s="3">
         <v>500126</v>
       </c>
-      <c r="B90" s="3" t="s">
+      <c r="B90" s="3">
+        <v>500126</v>
+      </c>
+      <c r="C90" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A91" s="3">
         <v>500132</v>
       </c>
-      <c r="B91" s="3" t="s">
+      <c r="B91" s="3">
+        <v>500132</v>
+      </c>
+      <c r="C91" s="3" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A92" s="4">
         <v>500134</v>
       </c>
-      <c r="B92" s="4" t="s">
+      <c r="B92" s="4">
+        <v>500134</v>
+      </c>
+      <c r="C92" s="4" t="s">
         <v>92</v>
       </c>
     </row>

</xml_diff>